<commit_message>
Rerun all scripts; remove template workbook and empty unused files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cms_medicare_adhd_older_americans/out/medicare_partd_stimulant_2019_2024.xlsx
+++ b/cms_medicare_adhd_older_americans/out/medicare_partd_stimulant_2019_2024.xlsx
@@ -293,13 +293,13 @@
     <t>Schedule II stimulant ingredients commonly used for ADHD; non-stimulants such as atomoxetine, guanfacine, clonidine, and viloxazine are excluded.</t>
   </si>
   <si>
-    <t>The public CMS drug-spending file includes all Part D beneficiaries, including some under 65. These totals must not be labeled 65+ spending.</t>
+    <t>The public CMS drug-spending file includes all Part D beneficiaries, including some under 65. These totals must not be labeled 65+ spending. For 65+ figures, see build_stimulant_prescribing_dataset.py (CMS Part D Prescribers by Geography and Drug, GE65_* fields).</t>
   </si>
   <si>
     <t>Gross drug cost includes Medicare, plan, beneficiary and other payments and does not subtract manufacturer rebates/price concessions.</t>
   </si>
   <si>
-    <t>Beneficiary counts are unique within a product row. Summing them across stimulant products double-counts beneficiaries using multiple products, so the class-level field is labeled Beneficiary_Product_Counts.</t>
+    <t>Beneficiary counts are unique within a product row. Summing them across stimulant products double-counts beneficiaries using multiple products, so the class-level field is labeled Beneficiary_Product_Counts. No public CMS file gives a unique count of stimulant users across products, for any age group.</t>
   </si>
   <si>
     <t>This CMS file reports dosage units, not days supplied. A different Part D prescriber dataset is needed for days supplied.</t>

</xml_diff>